<commit_message>
Bug fixes with param updates, mutant + fract_mut > 0.0 confirmed matching Python for G13D, assuming others match as well.
</commit_message>
<xml_diff>
--- a/RAS/data/kinetic_parameter_multipliers.xlsx
+++ b/RAS/data/kinetic_parameter_multipliers.xlsx
@@ -146,10 +146,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.000"/>
     <numFmt numFmtId="166" formatCode="#,##0.0000000"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0000000000"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -321,7 +322,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -358,43 +359,31 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -402,11 +391,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -674,12 +659,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O24"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="2" width="11.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="11.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="8" style="2" width="11.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="2" width="15.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="2" width="14.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="14.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="15.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="9" style="2" width="14.01"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -781,35 +769,27 @@
         <v>16</v>
       </c>
       <c r="B3" s="11" t="n">
-        <f aca="false">1.9/2.1</f>
         <v>0.904761904761905</v>
       </c>
       <c r="C3" s="11" t="n">
-        <f aca="false">9.7/1.2</f>
         <v>8.08333333333333</v>
       </c>
       <c r="D3" s="11" t="n">
-        <f aca="false">8.1/0.9</f>
         <v>9</v>
       </c>
       <c r="E3" s="9" t="n">
-        <f aca="false">244.9/0.51*(0.00011)/(0.0000000093*2300000)</f>
         <v>2.46945154873544</v>
       </c>
       <c r="F3" s="9" t="n">
-        <f aca="false">(244.9/0.51)*(0.00025)/(0.0000000069*2200000)</f>
         <v>7.90836756309902</v>
       </c>
-      <c r="G3" s="12" t="n">
-        <f aca="false">B3*m</f>
+      <c r="G3" s="11" t="n">
         <v>5.27777777777778E-005</v>
       </c>
       <c r="H3" s="11" t="n">
-        <f aca="false">10.7/8.9</f>
         <v>1.20224719101124</v>
       </c>
       <c r="I3" s="11" t="n">
-        <f aca="false">8.2/7.8</f>
         <v>1.05128205128205</v>
       </c>
       <c r="J3" s="9" t="n">
@@ -819,11 +799,9 @@
         <v>1</v>
       </c>
       <c r="L3" s="11" t="n">
-        <f aca="false">8.1/7.2</f>
         <v>1.125</v>
       </c>
-      <c r="M3" s="13" t="n">
-        <f aca="false">12.9/17.3</f>
+      <c r="M3" s="12" t="n">
         <v>0.745664739884393</v>
       </c>
       <c r="N3" s="9" t="n">
@@ -838,49 +816,42 @@
         <v>17</v>
       </c>
       <c r="B4" s="11" t="n">
-        <f aca="false">0.81/0.33</f>
         <v>2.45454545454545</v>
       </c>
       <c r="C4" s="11" t="n">
-        <f aca="false">13.5/1.2</f>
         <v>11.25</v>
       </c>
       <c r="D4" s="11" t="n">
-        <f aca="false">9.3/0.9</f>
         <v>10.3333333333333</v>
       </c>
-      <c r="E4" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="12" t="n">
-        <f aca="false">B4*m</f>
+      <c r="E4" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="11" t="n">
         <v>0.000143181818181818</v>
       </c>
       <c r="H4" s="11" t="n">
-        <f aca="false">13.8/8.9</f>
         <v>1.55056179775281</v>
       </c>
       <c r="I4" s="11" t="n">
-        <f aca="false">8.8/7.8</f>
         <v>1.12820512820513</v>
       </c>
-      <c r="J4" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="14" t="n">
+      <c r="J4" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="13" t="n">
         <v>1</v>
       </c>
       <c r="L4" s="11" t="n">
-        <f aca="false">8.4/7.2</f>
         <v>1.16666666666667</v>
       </c>
-      <c r="M4" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" s="14" t="n">
+      <c r="M4" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="13" t="n">
         <v>1</v>
       </c>
       <c r="O4" s="10" t="n">
@@ -891,16 +862,13 @@
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="15" t="n">
-        <f aca="false">2.4/10.2</f>
+      <c r="B5" s="14" t="n">
         <v>0.235294117647059</v>
       </c>
-      <c r="C5" s="15" t="n">
-        <f aca="false">4.4/0.79</f>
+      <c r="C5" s="14" t="n">
         <v>5.56962025316456</v>
       </c>
-      <c r="D5" s="15" t="n">
-        <f aca="false">2.8/2.3</f>
+      <c r="D5" s="14" t="n">
         <v>1.21739130434783</v>
       </c>
       <c r="E5" s="9" t="n">
@@ -909,8 +877,7 @@
       <c r="F5" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="16" t="n">
-        <f aca="false">B5*m</f>
+      <c r="G5" s="9" t="n">
         <v>1.37254901960784E-005</v>
       </c>
       <c r="H5" s="9" t="n">
@@ -990,50 +957,42 @@
         <v>20</v>
       </c>
       <c r="B7" s="11" t="n">
-        <f aca="false">0.5/2.1</f>
         <v>0.238095238095238</v>
       </c>
       <c r="C7" s="11" t="n">
-        <f aca="false">0.5/1.3</f>
         <v>0.384615384615385</v>
       </c>
       <c r="D7" s="11" t="n">
-        <f aca="false">0.9/0.9</f>
-        <v>1</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="12" t="n">
-        <f aca="false">B7*m</f>
+        <v>1</v>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="11" t="n">
         <v>1.38888888888889E-005</v>
       </c>
       <c r="H7" s="11" t="n">
-        <f aca="false">46.8/8.9</f>
         <v>5.25842696629213</v>
       </c>
       <c r="I7" s="11" t="n">
-        <f aca="false">7.3/7.8</f>
         <v>0.935897435897436</v>
       </c>
-      <c r="J7" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="14" t="n">
+      <c r="J7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="13" t="n">
         <v>1</v>
       </c>
       <c r="L7" s="11" t="n">
-        <f aca="false">7.5/7.2</f>
         <v>1.04166666666667</v>
       </c>
-      <c r="M7" s="17" t="n">
-        <f aca="false">127/56</f>
+      <c r="M7" s="15" t="n">
         <v>2.26785714285714</v>
       </c>
-      <c r="N7" s="14" t="n">
+      <c r="N7" s="13" t="n">
         <v>1</v>
       </c>
       <c r="O7" s="10" t="n">
@@ -1045,15 +1004,12 @@
         <v>21</v>
       </c>
       <c r="B8" s="11" t="n">
-        <f aca="false">1.8/2.1</f>
         <v>0.857142857142857</v>
       </c>
       <c r="C8" s="11" t="n">
-        <f aca="false">2.2/1.2</f>
         <v>1.83333333333333</v>
       </c>
       <c r="D8" s="11" t="n">
-        <f aca="false">0.6/0.9</f>
         <v>0.666666666666667</v>
       </c>
       <c r="E8" s="9" t="n">
@@ -1062,16 +1018,13 @@
       <c r="F8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="12" t="n">
-        <f aca="false">B8*m</f>
+      <c r="G8" s="11" t="n">
         <v>5E-005</v>
       </c>
       <c r="H8" s="11" t="n">
-        <f aca="false">12.3/8.9</f>
         <v>1.38202247191011</v>
       </c>
       <c r="I8" s="11" t="n">
-        <f aca="false">8.2/7.8</f>
         <v>1.05128205128205</v>
       </c>
       <c r="J8" s="9" t="n">
@@ -1081,11 +1034,9 @@
         <v>1</v>
       </c>
       <c r="L8" s="11" t="n">
-        <f aca="false">7.4/7.2</f>
         <v>1.02777777777778</v>
       </c>
-      <c r="M8" s="17" t="n">
-        <f aca="false">67/56</f>
+      <c r="M8" s="15" t="n">
         <v>1.19642857142857</v>
       </c>
       <c r="N8" s="9" t="n">
@@ -1100,35 +1051,27 @@
         <v>22</v>
       </c>
       <c r="B9" s="11" t="n">
-        <f aca="false">1.4/2.1</f>
         <v>0.666666666666667</v>
       </c>
       <c r="C9" s="11" t="n">
-        <f aca="false">1.6/1.2</f>
         <v>1.33333333333333</v>
       </c>
       <c r="D9" s="11" t="n">
-        <f aca="false">9.5/0.9</f>
         <v>10.5555555555556</v>
       </c>
       <c r="E9" s="9" t="n">
-        <f aca="false">0.7/0.51</f>
         <v>1.37254901960784</v>
       </c>
       <c r="F9" s="9" t="n">
-        <f aca="false">4.8/1.4</f>
         <v>3.42857142857143</v>
       </c>
-      <c r="G9" s="12" t="n">
-        <f aca="false">B9*m</f>
+      <c r="G9" s="11" t="n">
         <v>3.88888888888889E-005</v>
       </c>
       <c r="H9" s="11" t="n">
-        <f aca="false">4.8/8.9</f>
         <v>0.539325842696629</v>
       </c>
       <c r="I9" s="11" t="n">
-        <f aca="false">7/7.8</f>
         <v>0.897435897435898</v>
       </c>
       <c r="J9" s="9" t="n">
@@ -1138,11 +1081,9 @@
         <v>1</v>
       </c>
       <c r="L9" s="11" t="n">
-        <f aca="false">7.6/7.2</f>
         <v>1.05555555555556</v>
       </c>
-      <c r="M9" s="17" t="n">
-        <f aca="false">270/56</f>
+      <c r="M9" s="15" t="n">
         <v>4.82142857142857</v>
       </c>
       <c r="N9" s="9" t="n">
@@ -1157,49 +1098,42 @@
         <v>23</v>
       </c>
       <c r="B10" s="11" t="n">
-        <f aca="false">1.6/2.1</f>
         <v>0.761904761904762</v>
       </c>
       <c r="C10" s="11" t="n">
-        <f aca="false">1.5/1.2</f>
         <v>1.25</v>
       </c>
       <c r="D10" s="11" t="n">
-        <f aca="false">4.9/0.9</f>
         <v>5.44444444444445</v>
       </c>
-      <c r="E10" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="12" t="n">
-        <f aca="false">B10*m</f>
+      <c r="E10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="11" t="n">
         <v>4.44444444444444E-005</v>
       </c>
       <c r="H10" s="11" t="n">
-        <f aca="false">4.7/8.9</f>
         <v>0.528089887640449</v>
       </c>
       <c r="I10" s="11" t="n">
-        <f aca="false">7.5/7.8</f>
         <v>0.961538461538462</v>
       </c>
-      <c r="J10" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="14" t="n">
+      <c r="J10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="13" t="n">
         <v>1</v>
       </c>
       <c r="L10" s="11" t="n">
-        <f aca="false">8/7.2</f>
         <v>1.11111111111111</v>
       </c>
-      <c r="M10" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="N10" s="14" t="n">
+      <c r="M10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" s="13" t="n">
         <v>1</v>
       </c>
       <c r="O10" s="10" t="n">
@@ -1211,15 +1145,12 @@
         <v>24</v>
       </c>
       <c r="B11" s="9" t="n">
-        <f aca="false">0.043/0.028</f>
         <v>1.53571428571429</v>
       </c>
       <c r="C11" s="9" t="n">
-        <f aca="false">1.4/2</f>
         <v>0.7</v>
       </c>
       <c r="D11" s="9" t="n">
-        <f aca="false">13/11</f>
         <v>1.18181818181818</v>
       </c>
       <c r="E11" s="9" t="n">
@@ -1228,8 +1159,7 @@
       <c r="F11" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="16" t="n">
-        <f aca="false">0.09/10</f>
+      <c r="G11" s="9" t="n">
         <v>0.009</v>
       </c>
       <c r="H11" s="9" t="n">
@@ -1261,16 +1191,13 @@
       <c r="A12" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="17" t="n">
-        <f aca="false">1.8/68</f>
+      <c r="B12" s="15" t="n">
         <v>0.0264705882352941</v>
       </c>
       <c r="C12" s="9" t="n">
-        <f aca="false">0.37/0.79</f>
         <v>0.468354430379747</v>
       </c>
       <c r="D12" s="9" t="n">
-        <f aca="false">0.11/2.3</f>
         <v>0.0478260869565217</v>
       </c>
       <c r="E12" s="9" t="n">
@@ -1279,8 +1206,7 @@
       <c r="F12" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="18" t="n">
-        <f aca="false">B12*m</f>
+      <c r="G12" s="15" t="n">
         <v>1.54411764705882E-006</v>
       </c>
       <c r="H12" s="9" t="n">
@@ -1298,8 +1224,7 @@
       <c r="L12" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="M12" s="17" t="n">
-        <f aca="false">348/56</f>
+      <c r="M12" s="15" t="n">
         <v>6.21428571428571</v>
       </c>
       <c r="N12" s="9" t="n">
@@ -1314,49 +1239,42 @@
         <v>26</v>
       </c>
       <c r="B13" s="11" t="n">
-        <f aca="false">1.2/2.1</f>
         <v>0.571428571428571</v>
       </c>
       <c r="C13" s="11" t="n">
-        <f aca="false">4.8/1.2</f>
         <v>4</v>
       </c>
       <c r="D13" s="11" t="n">
-        <f aca="false">0.2/0.9</f>
         <v>0.222222222222222</v>
       </c>
-      <c r="E13" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="12" t="n">
-        <f aca="false">B13*m</f>
+      <c r="E13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="11" t="n">
         <v>3.33333333333333E-005</v>
       </c>
       <c r="H13" s="11" t="n">
-        <f aca="false">15.8/8.9</f>
         <v>1.7752808988764</v>
       </c>
       <c r="I13" s="11" t="n">
-        <f aca="false">8/7.8</f>
         <v>1.02564102564103</v>
       </c>
-      <c r="J13" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="14" t="n">
+      <c r="J13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="13" t="n">
         <v>1</v>
       </c>
       <c r="L13" s="11" t="n">
-        <f aca="false">7/7.2</f>
         <v>0.972222222222222</v>
       </c>
-      <c r="M13" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" s="14" t="n">
+      <c r="M13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" s="13" t="n">
         <v>1</v>
       </c>
       <c r="O13" s="10" t="n">
@@ -1368,35 +1286,27 @@
         <v>27</v>
       </c>
       <c r="B14" s="11" t="n">
-        <f aca="false">0.05/2.1</f>
         <v>0.0238095238095238</v>
       </c>
       <c r="C14" s="11" t="n">
-        <f aca="false">0.2/1.2</f>
         <v>0.166666666666667</v>
       </c>
       <c r="D14" s="11" t="n">
-        <f aca="false">0.9/0.9</f>
         <v>1</v>
       </c>
       <c r="E14" s="9" t="n">
-        <f aca="false">1.16/0.51</f>
         <v>2.27450980392157</v>
       </c>
       <c r="F14" s="9" t="n">
-        <f aca="false">5.8/1.4</f>
         <v>4.14285714285714</v>
       </c>
-      <c r="G14" s="12" t="n">
-        <f aca="false">B14*m</f>
+      <c r="G14" s="11" t="n">
         <v>1.38888888888889E-006</v>
       </c>
       <c r="H14" s="11" t="n">
-        <f aca="false">100/8.9</f>
         <v>11.2359550561798</v>
       </c>
       <c r="I14" s="11" t="n">
-        <f aca="false">7.1/7.8</f>
         <v>0.91025641025641</v>
       </c>
       <c r="J14" s="9" t="n">
@@ -1406,11 +1316,9 @@
         <v>1</v>
       </c>
       <c r="L14" s="11" t="n">
-        <f aca="false">7.5/7.2</f>
         <v>1.04166666666667</v>
       </c>
-      <c r="M14" s="17" t="n">
-        <f aca="false">411/56</f>
+      <c r="M14" s="15" t="n">
         <v>7.33928571428571</v>
       </c>
       <c r="N14" s="9" t="n">
@@ -1425,49 +1333,42 @@
         <v>28</v>
       </c>
       <c r="B15" s="11" t="n">
-        <f aca="false">1.1/2.1</f>
         <v>0.523809523809524</v>
       </c>
       <c r="C15" s="11" t="n">
-        <f aca="false">2.5/1.2</f>
         <v>2.08333333333333</v>
       </c>
       <c r="D15" s="11" t="n">
-        <f aca="false">0.8/0.9</f>
         <v>0.888888888888889</v>
       </c>
-      <c r="E15" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="12" t="n">
-        <f aca="false">B15*m</f>
+      <c r="E15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="11" t="n">
         <v>3.05555555555556E-005</v>
       </c>
       <c r="H15" s="11" t="n">
-        <f aca="false">26.6/8.9</f>
         <v>2.98876404494382</v>
       </c>
       <c r="I15" s="11" t="n">
-        <f aca="false">8.2/7.8</f>
         <v>1.05128205128205</v>
       </c>
-      <c r="J15" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="14" t="n">
+      <c r="J15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="13" t="n">
         <v>1</v>
       </c>
       <c r="L15" s="11" t="n">
-        <f aca="false">7.7/7.2</f>
         <v>1.06944444444444</v>
       </c>
-      <c r="M15" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="N15" s="14" t="n">
+      <c r="M15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" s="13" t="n">
         <v>1</v>
       </c>
       <c r="O15" s="10" t="n">
@@ -1479,15 +1380,12 @@
         <v>29</v>
       </c>
       <c r="B16" s="11" t="n">
-        <f aca="false">1.9/2.1</f>
         <v>0.904761904761905</v>
       </c>
       <c r="C16" s="11" t="n">
-        <f aca="false">1.6/1.2</f>
         <v>1.33333333333333</v>
       </c>
       <c r="D16" s="11" t="n">
-        <f aca="false">6.3/0.9</f>
         <v>7</v>
       </c>
       <c r="E16" s="9" t="n">
@@ -1496,16 +1394,13 @@
       <c r="F16" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="12" t="n">
-        <f aca="false">B16*m</f>
+      <c r="G16" s="11" t="n">
         <v>5.27777777777778E-005</v>
       </c>
       <c r="H16" s="11" t="n">
-        <f aca="false">5.2/8.9</f>
         <v>0.584269662921348</v>
       </c>
       <c r="I16" s="11" t="n">
-        <f aca="false">7/7.8</f>
         <v>0.897435897435898</v>
       </c>
       <c r="J16" s="9" t="n">
@@ -1515,11 +1410,9 @@
         <v>1</v>
       </c>
       <c r="L16" s="11" t="n">
-        <f aca="false">7.4/7.2</f>
         <v>1.02777777777778</v>
       </c>
-      <c r="M16" s="17" t="n">
-        <f aca="false">129/56</f>
+      <c r="M16" s="15" t="n">
         <v>2.30357142857143</v>
       </c>
       <c r="N16" s="9" t="n">
@@ -1534,15 +1427,12 @@
         <v>30</v>
       </c>
       <c r="B17" s="11" t="n">
-        <f aca="false">3.2/2.1</f>
         <v>1.52380952380952</v>
       </c>
       <c r="C17" s="11" t="n">
-        <f aca="false">3.6/1.2</f>
         <v>3</v>
       </c>
       <c r="D17" s="11" t="n">
-        <f aca="false">0.7/0.9</f>
         <v>0.777777777777778</v>
       </c>
       <c r="E17" s="9" t="n">
@@ -1551,16 +1441,13 @@
       <c r="F17" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="12" t="n">
-        <f aca="false">B17*m</f>
+      <c r="G17" s="11" t="n">
         <v>8.88888888888889E-005</v>
       </c>
       <c r="H17" s="11" t="n">
-        <f aca="false">19.6/8.9</f>
         <v>2.20224719101124</v>
       </c>
       <c r="I17" s="11" t="n">
-        <f aca="false">8.8/7.8</f>
         <v>1.12820512820513</v>
       </c>
       <c r="J17" s="9" t="n">
@@ -1570,7 +1457,6 @@
         <v>1</v>
       </c>
       <c r="L17" s="11" t="n">
-        <f aca="false">8.2/7.2</f>
         <v>1.13888888888889</v>
       </c>
       <c r="M17" s="9" t="n">
@@ -1588,15 +1474,12 @@
         <v>31</v>
       </c>
       <c r="B18" s="11" t="n">
-        <f aca="false">2/2.1</f>
         <v>0.952380952380952</v>
       </c>
       <c r="C18" s="11" t="n">
-        <f aca="false">3.4/1.2</f>
         <v>2.83333333333333</v>
       </c>
       <c r="D18" s="11" t="n">
-        <f aca="false">1.2/0.9</f>
         <v>1.33333333333333</v>
       </c>
       <c r="E18" s="9" t="n">
@@ -1605,16 +1488,13 @@
       <c r="F18" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G18" s="12" t="n">
-        <f aca="false">B18*m</f>
+      <c r="G18" s="11" t="n">
         <v>5.55555555555556E-005</v>
       </c>
       <c r="H18" s="11" t="n">
-        <f aca="false">87/8.9</f>
         <v>9.77528089887641</v>
       </c>
       <c r="I18" s="11" t="n">
-        <f aca="false">7.9/7.8</f>
         <v>1.01282051282051</v>
       </c>
       <c r="J18" s="9" t="n">
@@ -1624,7 +1504,6 @@
         <v>1</v>
       </c>
       <c r="L18" s="11" t="n">
-        <f aca="false">7.4/7.2</f>
         <v>1.02777777777778</v>
       </c>
       <c r="M18" s="9" t="n">
@@ -1642,15 +1521,12 @@
         <v>32</v>
       </c>
       <c r="B19" s="9" t="n">
-        <f aca="false">1.83/20.93</f>
         <v>0.0874343048256092</v>
       </c>
       <c r="C19" s="9" t="n">
-        <f aca="false">9.6/6.5</f>
         <v>1.47692307692308</v>
       </c>
       <c r="D19" s="9" t="n">
-        <f aca="false">9.2/15</f>
         <v>0.613333333333333</v>
       </c>
       <c r="E19" s="9" t="n">
@@ -1659,12 +1535,10 @@
       <c r="F19" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="16" t="n">
-        <f aca="false">B19*m</f>
+      <c r="G19" s="9" t="n">
         <v>5.10033444816054E-006</v>
       </c>
       <c r="H19" s="9" t="n">
-        <f aca="false">25/35</f>
         <v>0.714285714285714</v>
       </c>
       <c r="I19" s="9" t="n">
@@ -1694,15 +1568,12 @@
         <v>33</v>
       </c>
       <c r="B20" s="9" t="n">
-        <f aca="false">0.348/20.93</f>
         <v>0.0166268514094601</v>
       </c>
       <c r="C20" s="9" t="n">
-        <f aca="false">9.1/6.5</f>
         <v>1.4</v>
       </c>
       <c r="D20" s="9" t="n">
-        <f aca="false">9/15</f>
         <v>0.6</v>
       </c>
       <c r="E20" s="9" t="n">
@@ -1711,12 +1582,10 @@
       <c r="F20" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="16" t="n">
-        <f aca="false">B20*m</f>
+      <c r="G20" s="9" t="n">
         <v>9.69899665551839E-007</v>
       </c>
       <c r="H20" s="9" t="n">
-        <f aca="false">2000/35</f>
         <v>57.1428571428571</v>
       </c>
       <c r="I20" s="9" t="n">
@@ -1746,30 +1615,24 @@
         <v>34</v>
       </c>
       <c r="B21" s="9" t="n">
-        <f aca="false">0.455/20.93</f>
         <v>0.0217391304347826</v>
       </c>
       <c r="C21" s="9" t="n">
-        <f aca="false">16/6.5</f>
         <v>2.46153846153846</v>
       </c>
       <c r="D21" s="9" t="n">
-        <f aca="false">16/15</f>
         <v>1.06666666666667</v>
       </c>
       <c r="E21" s="9" t="n">
-        <f aca="false">1</f>
         <v>1</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="16" t="n">
-        <f aca="false">B21*m</f>
+      <c r="G21" s="9" t="n">
         <v>1.26811594202899E-006</v>
       </c>
       <c r="H21" s="9" t="n">
-        <f aca="false">2/35</f>
         <v>0.0571428571428571</v>
       </c>
       <c r="I21" s="9" t="n">
@@ -1784,8 +1647,7 @@
       <c r="L21" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="M21" s="17" t="n">
-        <f aca="false">134/56</f>
+      <c r="M21" s="15" t="n">
         <v>2.39285714285714</v>
       </c>
       <c r="N21" s="9" t="n">
@@ -1800,30 +1662,24 @@
         <v>35</v>
       </c>
       <c r="B22" s="9" t="n">
-        <f aca="false">1.63/20.93</f>
         <v>0.0778786430960344</v>
       </c>
       <c r="C22" s="9" t="n">
-        <f aca="false">6.8/6.5</f>
         <v>1.04615384615385</v>
       </c>
       <c r="D22" s="9" t="n">
-        <f aca="false">19/15</f>
         <v>1.26666666666667</v>
       </c>
       <c r="E22" s="9" t="n">
-        <f aca="false">1</f>
         <v>1</v>
       </c>
       <c r="F22" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="16" t="n">
-        <f aca="false">B22*m</f>
+      <c r="G22" s="9" t="n">
         <v>4.54292084726867E-006</v>
       </c>
       <c r="H22" s="9" t="n">
-        <f aca="false">50/35</f>
         <v>1.42857142857143</v>
       </c>
       <c r="I22" s="9" t="n">
@@ -1853,15 +1709,12 @@
         <v>36</v>
       </c>
       <c r="B23" s="9" t="n">
-        <f aca="false">0.366/20.93</f>
         <v>0.0174868609651218</v>
       </c>
       <c r="C23" s="9" t="n">
-        <f aca="false">7.4/6.5</f>
         <v>1.13846153846154</v>
       </c>
       <c r="D23" s="9" t="n">
-        <f aca="false">6.7/15</f>
         <v>0.446666666666667</v>
       </c>
       <c r="E23" s="9" t="n">
@@ -1870,12 +1723,10 @@
       <c r="F23" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="16" t="n">
-        <f aca="false">B23*m</f>
+      <c r="G23" s="9" t="n">
         <v>1.02006688963211E-006</v>
       </c>
       <c r="H23" s="9" t="n">
-        <f aca="false">1500/35</f>
         <v>42.8571428571429</v>
       </c>
       <c r="I23" s="9" t="n">
@@ -1901,52 +1752,46 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="20" t="n">
-        <f aca="false">1.52/20.93</f>
+      <c r="B24" s="17" t="n">
         <v>0.0726230291447683</v>
       </c>
-      <c r="C24" s="20" t="n">
-        <f aca="false">6.5/6.5</f>
-        <v>1</v>
-      </c>
-      <c r="D24" s="20" t="n">
-        <f aca="false">12/15</f>
+      <c r="C24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="E24" s="20" t="n">
-        <f aca="false">1</f>
-        <v>1</v>
-      </c>
-      <c r="F24" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="21" t="n">
-        <f aca="false">B24*m</f>
+      <c r="E24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="17" t="n">
         <v>4.23634336677815E-006</v>
       </c>
-      <c r="H24" s="20" t="n">
-        <f aca="false">100/35</f>
+      <c r="H24" s="17" t="n">
         <v>2.85714285714286</v>
       </c>
-      <c r="I24" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="K24" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="M24" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="N24" s="20" t="n">
+      <c r="I24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" s="17" t="n">
         <v>1</v>
       </c>
       <c r="O24" s="10" t="n">

</xml_diff>

<commit_message>
tricomplex model working with drugs.
</commit_message>
<xml_diff>
--- a/RAS/data/kinetic_parameter_multipliers.xlsx
+++ b/RAS/data/kinetic_parameter_multipliers.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="BaseParams" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="TricomplexParams" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
   <definedNames>
     <definedName function="false" hidden="false" name="m" vbProcedure="false">'[1]WT and Mutant multipliers'!$Q$5</definedName>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="43">
   <si>
     <t xml:space="preserve">KRAS WT or Mutant</t>
   </si>
@@ -140,6 +141,21 @@
   </si>
   <si>
     <t xml:space="preserve">Q61W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K_D_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full confidence interval is 108-158</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full confidence interval is 307-432</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full confidence interval is 136-174</t>
   </si>
 </sst>
 </file>
@@ -152,7 +168,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.0000000"/>
     <numFmt numFmtId="167" formatCode="#,##0.0000000000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,6 +195,14 @@
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -322,7 +346,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -393,6 +417,18 @@
     </xf>
     <xf numFmtId="167" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1807,4 +1843,71 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="39.71"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>154</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>131</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>364</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>